<commit_message>
Actualización automática 2026-02-05 15:30:14
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>462.67</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2 de 25</t>
+          <t>3 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2491,7 +2491,7 @@
         <v>767.9400000000001</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>462.67</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
         <v>10012.66</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>5714.320000000001</v>
+        <v>6176.990000000001</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>38870</v>
@@ -3225,13 +3225,13 @@
         <v>39250</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4798.48</v>
+        <v>5261.15</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34451.52</v>
+        <v>33988.85</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1222542675159236</v>
+        <v>0.1340420382165605</v>
       </c>
     </row>
     <row r="14">
@@ -3292,13 +3292,13 @@
         <v>45934.313</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5714.32</v>
+        <v>6176.99</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40219.99299999999</v>
+        <v>39757.323</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1244019911650796</v>
+        <v>0.1344744178496803</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-03 14:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>325.63</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0 de 25</t>
+          <t>1 de 25</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2159,7 +2159,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2788,7 +2788,7 @@
         <v>-142.56</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>325.63</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>1000</v>
@@ -2886,7 +2886,7 @@
         <v>50050.21</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0</v>
+        <v>325.63</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>38870</v>

</xml_diff>

<commit_message>
Actualización automática 2026-03-11 17:30:22
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1089,7 +1089,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>0</v>
+        <v>396.6</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>0</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>396.58</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -2111,22 +2111,22 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
+          <t>1 de 25</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
           <t>0 de 25</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>0 de 25</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>0 de 25</t>
+          <t>1 de 25</t>
         </is>
       </c>
       <c r="Q27" s="4" t="inlineStr">
@@ -2437,7 +2437,7 @@
         <v>5376.52</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>396.6</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>1500</v>
@@ -2491,7 +2491,7 @@
         <v>484.7</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>396.58</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
         <v>50050.21</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>325.63</v>
+        <v>1118.81</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>38870</v>
@@ -2911,7 +2911,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3105,13 +3105,13 @@
         <v>250</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>396.6</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>250</v>
+        <v>-146.6</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>1.5864</v>
       </c>
     </row>
     <row r="9">
@@ -3225,13 +3225,13 @@
         <v>68268</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>396.58</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>68268</v>
+        <v>67871.42</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.005809163883517899</v>
       </c>
     </row>
     <row r="14">
@@ -3268,13 +3268,13 @@
         <v>74230.31300000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>325.63</v>
+        <v>1118.81</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>73904.683</v>
+        <v>73111.503</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.004386752350081024</v>
+        <v>0.01507214444858935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-17 08:30:22
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>5382.95</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>1 de 25</t>
+          <t>2 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2518,7 +2518,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>5382.95</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>12870</v>
@@ -2886,7 +2886,7 @@
         <v>56394.77</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>-5399.65</v>
+        <v>-16.70000000000022</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>38870</v>
@@ -2909,9 +2909,9 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3201,13 +3201,13 @@
         <v>39250</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-5950.28</v>
+        <v>-567.33</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>45200.28</v>
+        <v>39817.33</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.1515994904458599</v>
+        <v>-0.01445426751592357</v>
       </c>
     </row>
     <row r="13">
@@ -3268,13 +3268,13 @@
         <v>44110.233</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>-5399.65</v>
+        <v>-16.70000000000005</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>49509.88299999999</v>
+        <v>44126.933</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.1224126383553676</v>
+        <v>-0.0003785969573092041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-07 16:30:19
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -600,7 +600,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>63.92</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>356.4</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0</v>
@@ -1920,7 +1920,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>394.63</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2331,27 +2331,27 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="L31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>2 de 29</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -2399,7 +2399,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2488,7 +2488,7 @@
         <v>103.94</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>63.92</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
@@ -2974,7 +2974,7 @@
         <v>-7097.63</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>356.4</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1000</v>
@@ -3379,7 +3379,7 @@
         <v>131.05</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>394.63</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>500</v>
@@ -3585,7 +3585,7 @@
         <v>-786.5600000000002</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>0</v>
+        <v>814.9499999999999</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>38870</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-13 13:30:24
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>939.08</v>
+        <v>976.35</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2893,7 +2893,7 @@
         <v>5382.95</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>939.08</v>
+        <v>976.35</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>12870</v>
@@ -3585,7 +3585,7 @@
         <v>-786.5600000000002</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>1754.03</v>
+        <v>1791.3</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>38870</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-25 08:30:23
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VELASCO SAMANIEGO JIMMY FABRICIO</t>
+          <t>VELASQUEZ ARELLANO SAIRA MAGDALENA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VELASQUEZ ARELLANO SAIRA MAGDALENA</t>
+          <t>VIDAL VARGAS ANDREA DOMINIQUE</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VIDAL VARGAS ANDREA DOMINIQUE</t>
+          <t>ZAMBRANO ANGELA MARIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2157,10 +2157,10 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>146.97</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>16853.73</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ZAMBRANO ANGELA MARIA</t>
+          <t>ZAMBRANO ZAMBRANO JOSE ALEJANDRO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2217,10 +2217,10 @@
         <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>146.97</v>
+        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>16853.73</v>
+        <v>0</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2239,144 +2239,84 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ZAMBRANO ZAMBRANO JOSE ALEJANDRO</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>6 de 29</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="P31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="Q31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="R31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>1 de 28</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>1 de 28</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>6 de 28</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="R30" s="4" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-22 14:30:19
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -2088,7 +2088,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0</v>
+        <v>289.94</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0</v>
@@ -2100,10 +2100,10 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>8339.67</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>914.4</v>
       </c>
       <c r="O27" s="2" t="n">
         <v>0</v>
@@ -2391,32 +2391,32 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr">
         <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>0 de 30</t>
+          <t>1 de 30</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>0 de 30</t>
+          <t>1 de 30</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3520,7 +3520,7 @@
         <v>294.49</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>9544.01</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0</v>
@@ -3699,7 +3699,7 @@
         <v>64997.6</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>0</v>
+        <v>9544.01</v>
       </c>
       <c r="G46" s="6" t="n">
         <v>41650</v>
@@ -3722,9 +3722,9 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3870,13 +3870,13 @@
         <v>312</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>289.94</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>312</v>
+        <v>22.06</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>0.9292948717948718</v>
       </c>
     </row>
     <row r="7">
@@ -3990,13 +3990,13 @@
         <v>38234</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>8339.67</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>38234</v>
+        <v>29894.33</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.2181218287388189</v>
       </c>
     </row>
     <row r="12">
@@ -4014,13 +4014,13 @@
         <v>570</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>914.4</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>570</v>
+        <v>-344.4</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>1.60421052631579</v>
       </c>
     </row>
     <row r="13">
@@ -4033,13 +4033,13 @@
         <v>43267.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>9544.01</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>43267.5</v>
+        <v>33723.49</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.2205814988155082</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-31 08:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>-16.52</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -2812,7 +2812,7 @@
         <v>3425.52</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>-16.52</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2000</v>
@@ -3261,7 +3261,7 @@
         <v>16577.79</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>1219.72</v>
+        <v>1203.2</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>41650</v>
@@ -3286,7 +3286,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3576,13 +3576,13 @@
         <v>29057</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>-16.52</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>29057</v>
+        <v>29073.52</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>-0.0005685377017586124</v>
       </c>
     </row>
     <row r="13">
@@ -3619,13 +3619,13 @@
         <v>34779.313</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1219.72</v>
+        <v>1203.2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>33559.593</v>
+        <v>33576.113</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.03507027295220006</v>
+        <v>0.03459527794582946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-31 14:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -993,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>1462.41</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>1219.72</v>
+        <v>3397.8</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>0</v>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>0</v>
+        <v>453.18</v>
       </c>
       <c r="Q11" s="2" t="n">
         <v>0</v>
@@ -1413,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>987.15</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>644.64</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1713,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>6266.67</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>13307.98</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2306,67 +2306,67 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
+          <t>3 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>2 de 29</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="P31" s="4" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
         </is>
       </c>
       <c r="Q31" s="4" t="inlineStr">
@@ -2399,7 +2399,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2650,7 +2650,7 @@
         <v>2297.69</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>1462.41</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -2704,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1219.72</v>
+        <v>3850.98</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>3000</v>
@@ -2839,7 +2839,7 @@
         <v>189.57</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>1830.03</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3000</v>
@@ -3001,7 +3001,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>19574.65</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -3261,7 +3261,7 @@
         <v>16577.79</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>1203.2</v>
+        <v>26701.55</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>41650</v>
@@ -3285,8 +3285,8 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3360,13 +3360,13 @@
         <v>3800</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>8716.23</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3800</v>
+        <v>-4916.23</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>2.293744736842105</v>
       </c>
     </row>
     <row r="4">
@@ -3456,13 +3456,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>453.18</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>250</v>
+        <v>-203.18</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1.81272</v>
       </c>
     </row>
     <row r="8">
@@ -3528,13 +3528,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>198.24</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>115</v>
+        <v>-83.24000000000001</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>1.723826086956522</v>
       </c>
     </row>
     <row r="11">
@@ -3552,13 +3552,13 @@
         <v>254</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1219.72</v>
+        <v>3397.8</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-965.72</v>
+        <v>-3143.8</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4.802047244094489</v>
+        <v>13.37716535433071</v>
       </c>
     </row>
     <row r="12">
@@ -3576,13 +3576,13 @@
         <v>29057</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-16.52</v>
+        <v>13936.1</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>29073.52</v>
+        <v>15120.9</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0005685377017586124</v>
+        <v>0.479612485803765</v>
       </c>
     </row>
     <row r="13">
@@ -3619,13 +3619,13 @@
         <v>34779.313</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1203.2</v>
+        <v>26701.55</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>33576.113</v>
+        <v>8077.763</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.03459527794582946</v>
+        <v>0.7677423070432703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-13 14:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>0</v>
+        <v>169.3</v>
       </c>
       <c r="M26" s="2" t="n">
         <v>0</v>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>1 de 29</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
@@ -3136,7 +3136,7 @@
         <v>738.77</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>169.3</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>8000</v>
@@ -3261,7 +3261,7 @@
         <v>34614.9</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>-566.27</v>
+        <v>-396.97</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>41650</v>
@@ -3576,13 +3576,13 @@
         <v>960</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>169.3</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>960</v>
+        <v>790.7</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>0.1763541666666667</v>
       </c>
     </row>
     <row r="13">
@@ -3643,13 +3643,13 @@
         <v>42365.443</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>-566.27</v>
+        <v>-396.97</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42931.713</v>
+        <v>42762.413</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0.01336631839303557</v>
+        <v>-0.009370136882553075</v>
       </c>
     </row>
   </sheetData>

</xml_diff>